<commit_message>
Guardar cambios locales antes de integrar origin/main
</commit_message>
<xml_diff>
--- a/Part2_analyses/All_stats_clean.xlsx
+++ b/Part2_analyses/All_stats_clean.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\EHI_laterality\Part2_analyses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{232898B4-404D-42AF-91AE-692EE252C7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BCC5936-6915-4CE1-8502-09427CA3AF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7155" yWindow="-13980" windowWidth="19425" windowHeight="10305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="485">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="486">
   <si>
     <t>Regarding age</t>
   </si>
@@ -1484,6 +1484,9 @@
   </si>
   <si>
     <t>Repeat discarding people with no age or no sex</t>
+  </si>
+  <si>
+    <t>Controls NRH</t>
   </si>
 </sst>
 </file>
@@ -1741,7 +1744,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1863,6 +1866,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2384,18 +2390,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:S19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.26953125" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:19" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="40" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="22" t="s">
         <v>110</v>
@@ -2403,24 +2410,27 @@
       <c r="C3" s="22"/>
       <c r="D3" s="22"/>
       <c r="E3" s="22"/>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="22"/>
+      <c r="G3" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
       <c r="M3" s="11"/>
-      <c r="N3" s="60" t="s">
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="60"/>
-    </row>
-    <row r="4" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="R3" s="60"/>
+    </row>
+    <row r="4" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
@@ -2434,43 +2444,52 @@
         <v>62</v>
       </c>
       <c r="E4" s="23" t="s">
+        <v>485</v>
+      </c>
+      <c r="F4" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="L4" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="K4" s="12" t="s">
+      <c r="M4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="L4" s="12" t="s">
+      <c r="N4" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="O4" s="12" t="s">
+        <v>485</v>
+      </c>
+      <c r="P4" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="Q4" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="15" t="s">
+      <c r="R4" s="15" t="s">
         <v>471</v>
       </c>
-      <c r="P4" s="15" t="s">
+      <c r="S4" s="15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>0</v>
       </c>
@@ -2483,44 +2502,49 @@
       <c r="D5" s="24" t="s">
         <v>149</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="24">
+        <v>119</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="J5" s="9"/>
+      <c r="K5" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="J5" s="13" t="s">
+      <c r="L5" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="M5" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="N5" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="M5" s="13" t="s">
+      <c r="O5" s="13"/>
+      <c r="P5" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="N5" t="s">
-        <v>23</v>
-      </c>
-      <c r="O5" t="s">
-        <v>23</v>
-      </c>
-      <c r="P5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R5" t="s">
+        <v>23</v>
+      </c>
+      <c r="S5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>24</v>
       </c>
@@ -2533,44 +2557,49 @@
       <c r="D6" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="24">
+        <v>137</v>
+      </c>
+      <c r="F6" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="I6" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="J6" s="9"/>
+      <c r="K6" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J6" s="13" t="s">
+      <c r="L6" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="M6" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="L6" s="13" t="s">
+      <c r="N6" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="M6" s="13" t="s">
+      <c r="O6" s="13"/>
+      <c r="P6" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="N6" t="s">
-        <v>23</v>
-      </c>
-      <c r="O6" t="s">
-        <v>23</v>
-      </c>
-      <c r="P6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="Q6" t="s">
+        <v>23</v>
+      </c>
+      <c r="R6" t="s">
+        <v>23</v>
+      </c>
+      <c r="S6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>33</v>
       </c>
@@ -2583,44 +2612,49 @@
       <c r="D7" s="24" t="s">
         <v>153</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="24">
+        <v>178</v>
+      </c>
+      <c r="F7" s="24" t="s">
         <v>154</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="H7" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="J7" s="9"/>
+      <c r="K7" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="L7" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="M7" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="L7" s="13" t="s">
+      <c r="N7" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="M7" s="13" t="s">
+      <c r="O7" s="13"/>
+      <c r="P7" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="N7" t="s">
-        <v>23</v>
-      </c>
-      <c r="O7" s="10">
+      <c r="Q7" t="s">
+        <v>23</v>
+      </c>
+      <c r="R7" s="10">
         <v>3.61E-2</v>
       </c>
-      <c r="P7" s="10">
+      <c r="S7" s="10">
         <v>1.627E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>42</v>
       </c>
@@ -2633,44 +2667,49 @@
       <c r="D8" s="24" t="s">
         <v>157</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="24">
+        <v>450</v>
+      </c>
+      <c r="F8" s="24" t="s">
         <v>158</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="G8" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="H8" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="I8" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="J8" s="9"/>
+      <c r="K8" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="13" t="s">
+      <c r="L8" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="M8" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="N8" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="O8" s="13"/>
+      <c r="P8" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="N8" t="s">
-        <v>23</v>
-      </c>
-      <c r="O8" s="10">
+      <c r="Q8" t="s">
+        <v>23</v>
+      </c>
+      <c r="R8" s="10">
         <v>3.97E-4</v>
       </c>
-      <c r="P8" s="16">
+      <c r="S8" s="16">
         <v>8.5870000000000003E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>51</v>
       </c>
@@ -2683,52 +2722,57 @@
       <c r="D9" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="24">
+        <v>788</v>
+      </c>
+      <c r="F9" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="J9" s="9"/>
+      <c r="K9" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="O9" s="13"/>
+      <c r="P9" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="N9" t="s">
-        <v>23</v>
-      </c>
-      <c r="O9" s="10">
+      <c r="Q9" t="s">
+        <v>23</v>
+      </c>
+      <c r="R9" s="10">
         <v>6.7000000000000002E-4</v>
       </c>
-      <c r="P9" s="16">
+      <c r="S9" s="16">
         <v>3.8999999999999999E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="O10" s="10"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="R10" s="10"/>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="2" t="s">
         <v>1</v>
@@ -2736,18 +2780,20 @@
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="2"/>
+      <c r="G13" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="59" t="s">
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="K13" s="59"/>
-    </row>
-    <row r="14" spans="1:16" ht="58" x14ac:dyDescent="0.35">
+      <c r="M13" s="59"/>
+    </row>
+    <row r="14" spans="1:19" ht="58" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>4</v>
       </c>
@@ -2760,32 +2806,35 @@
       <c r="D14" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="5"/>
+      <c r="F14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="J14" s="6"/>
+      <c r="K14" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="L14" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="M14" s="7" t="s">
         <v>471</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="N14" s="7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="O14" s="68"/>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>0</v>
       </c>
@@ -2798,32 +2847,34 @@
       <c r="D15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="8"/>
+      <c r="F15" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="G15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="H15" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="I15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I15" s="9" t="s">
+      <c r="J15" s="9"/>
+      <c r="K15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="J15" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" t="s">
-        <v>23</v>
-      </c>
       <c r="L15" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M15" t="s">
+        <v>23</v>
+      </c>
+      <c r="N15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
@@ -2836,32 +2887,34 @@
       <c r="D16" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="8"/>
+      <c r="F16" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="G16" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="H16" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="I16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="I16" s="9" t="s">
+      <c r="J16" s="9"/>
+      <c r="K16" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="J16" t="s">
-        <v>23</v>
-      </c>
-      <c r="K16" t="s">
-        <v>23</v>
-      </c>
       <c r="L16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>33</v>
       </c>
@@ -2874,32 +2927,34 @@
       <c r="D17" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="8"/>
+      <c r="F17" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="G17" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="G17" s="9" t="s">
+      <c r="H17" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="I17" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I17" s="9" t="s">
+      <c r="J17" s="9"/>
+      <c r="K17" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="J17" t="s">
-        <v>23</v>
-      </c>
-      <c r="K17" t="s">
-        <v>23</v>
-      </c>
       <c r="L17" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M17" t="s">
+        <v>23</v>
+      </c>
+      <c r="N17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>42</v>
       </c>
@@ -2912,32 +2967,35 @@
       <c r="D18" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="8"/>
+      <c r="F18" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="H18" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="I18" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I18" s="9" t="s">
+      <c r="J18" s="9"/>
+      <c r="K18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="J18" t="s">
-        <v>23</v>
-      </c>
-      <c r="K18" s="10">
+      <c r="L18" t="s">
+        <v>23</v>
+      </c>
+      <c r="M18" s="10">
         <v>9.7999999999999997E-3</v>
       </c>
-      <c r="L18" s="10">
+      <c r="N18" s="10">
         <v>1.2710000000000001E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="O18" s="10"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>51</v>
       </c>
@@ -2950,35 +3008,38 @@
       <c r="D19" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="8"/>
+      <c r="F19" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="G19" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="H19" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="I19" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="J19" s="9"/>
+      <c r="K19" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="J19" t="s">
-        <v>23</v>
-      </c>
-      <c r="K19" s="10">
+      <c r="L19" t="s">
+        <v>23</v>
+      </c>
+      <c r="M19" s="10">
         <v>4.2739999999999998E-8</v>
       </c>
-      <c r="L19" s="10">
+      <c r="N19" s="10">
         <v>1.7499999999999999E-7</v>
       </c>
+      <c r="O19" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="Q3:R3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4396,7 +4457,7 @@
       </c>
       <c r="K30" s="65"/>
     </row>
-    <row r="31" spans="1:18" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="58" x14ac:dyDescent="0.35">
       <c r="B31" s="45" t="s">
         <v>482</v>
       </c>

</xml_diff>